<commit_message>
artifacts: publish E0016 output
</commit_message>
<xml_diff>
--- a/outputs/experiment_registry_excel_20260828/HCP_dFC_实验登记册.xlsx
+++ b/outputs/experiment_registry_excel_20260828/HCP_dFC_实验登记册.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R63312fcc803f4112"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实验登记" sheetId="2" r:id="Rbbcaa5cb9a3a4ce4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="Rcf1340f4d01c4648"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R3c09f4b126e746b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实验登记" sheetId="2" r:id="Re5667b84fe554379"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="R26c875b4db5a47e9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -701,7 +701,7 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="B5" s="15" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -709,7 +709,7 @@
         <x:v>计划中</x:v>
       </x:c>
       <x:c r="B6" s="15" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -717,7 +717,7 @@
         <x:v>等待结论</x:v>
       </x:c>
       <x:c r="B7" s="15" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -725,7 +725,7 @@
         <x:v>最新登记日期</x:v>
       </x:c>
       <x:c r="B8" s="18" t="n">
-        <x:v>46262.416666666664</x:v>
+        <x:v>46265.11111111111</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3212,7 +3212,7 @@
         <x:v>sequence</x:v>
       </x:c>
       <x:c r="E19" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>AWAITING_CONCLUSION</x:v>
       </x:c>
       <x:c r="F19" s="53" t="n">
         <x:v>46262.37152777778</x:v>
@@ -3309,27 +3309,47 @@
       <x:c r="AN19" t="str">
         <x:v>objective_loss</x:v>
       </x:c>
-      <x:c r="AO19" s="55"/>
-      <x:c r="AP19" s="55"/>
-      <x:c r="AQ19" s="55"/>
-      <x:c r="AR19" s="55"/>
-      <x:c r="AS19" s="55"/>
-      <x:c r="AT19" s="55"/>
-      <x:c r="AU19" s="55"/>
-      <x:c r="AV19" s="55"/>
-      <x:c r="AW19" s="55"/>
-      <x:c r="AX19" s="55"/>
+      <x:c r="AO19" s="55" t="n">
+        <x:v>0.028340847479014455</x:v>
+      </x:c>
+      <x:c r="AP19" s="55" t="str">
+        <x:v>E0016-s42-20260831T021312Z-72286c1</x:v>
+      </x:c>
+      <x:c r="AQ19" s="55" t="str">
+        <x:v>COMPLETED</x:v>
+      </x:c>
+      <x:c r="AR19" s="55" t="n">
+        <x:v>1.9668978845016867</x:v>
+      </x:c>
+      <x:c r="AS19" s="55" t="n">
+        <x:v>0.4810664133180546</x:v>
+      </x:c>
+      <x:c r="AT19" s="55" t="n">
+        <x:v>-0.009806781289200121</x:v>
+      </x:c>
+      <x:c r="AU19" s="55" t="n">
+        <x:v>0.009446948578086081</x:v>
+      </x:c>
+      <x:c r="AV19" s="55" t="n">
+        <x:v>0.1298238670901407</x:v>
+      </x:c>
+      <x:c r="AW19" s="55" t="n">
+        <x:v>0.09584946572026119</x:v>
+      </x:c>
+      <x:c r="AX19" s="55" t="n">
+        <x:v>0.23595558293016416</x:v>
+      </x:c>
       <x:c r="AY19" t="str">
-        <x:v>计划中：拆分E0012的两项动态损失，以识别时间方向与幅值校准的独立贡献。</x:v>
+        <x:v>训练、验证与动态审计已完成：差分标准差比中位数全程0.00843、non-overlap 0.00258，长程残差相关−0.00981；单独L_diff未解除动态塌缩。</x:v>
       </x:c>
       <x:c r="AZ19" t="str">
-        <x:v>运行 seed=42 后执行验证集评估和动态审计；仅与E0012作验证集比较。</x:v>
+        <x:v>与E0012、E0017在验证集比较，判断L_diff与L_var的协同是否必要。</x:v>
       </x:c>
       <x:c r="BA19" t="str">
         <x:v>configs/experiments/E0016_gcn_gru_difference_only_mse_v1.yaml</x:v>
       </x:c>
       <x:c r="BB19" t="str">
-        <x:v>fd48785e9c6fcd1b35b3c782fe4cb4fa1f4bcd10cdb078e9d23b51e985324242</x:v>
+        <x:v>ede3bf1898d10e3192957dee47e5deddd3de2c4df9c1f0e992f6d0ff762f9b64</x:v>
       </x:c>
       <x:c r="BC19" t="str">
         <x:v>固定完成50个epoch，仅在验证集运行动态审计且不查看测试集；与E0012比较差分时间相关、差分标准差比和频段功率比。若变化方向改善但幅值/功率仍失配，说明L_diff主要提供时间方向而不足以校准幅值。</x:v>
@@ -3486,7 +3506,7 @@
         <x:v>configs/experiments/E0017_gcn_gru_variance_only_mse_v1.yaml</x:v>
       </x:c>
       <x:c r="BB20" t="str">
-        <x:v>605b4baa9edfb27aae383ab56f6cda6e5adec41951e05db1d7d55099e7f21b35</x:v>
+        <x:v>5b8511feaa9d49db67144b3e97e39dd76c2c7eefdaedc59f8749b61764d419d7</x:v>
       </x:c>
       <x:c r="BC20" t="str">
         <x:v>固定完成50个epoch，仅在验证集运行动态审计且不查看测试集；与E0012比较差分标准差比、低/中频功率比和差分时间相关。若幅值改善而时间相关仍低，说明L_var主要校准振幅而不能恢复时间细节。</x:v>
@@ -5850,7 +5870,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb61b6d2439d4eaf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R973a768845d14348"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
artifacts: publish E0018 loss-scale control
</commit_message>
<xml_diff>
--- a/outputs/experiment_registry_excel_20260828/HCP_dFC_实验登记册.xlsx
+++ b/outputs/experiment_registry_excel_20260828/HCP_dFC_实验登记册.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R3c09f4b126e746b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实验登记" sheetId="2" r:id="Re5667b84fe554379"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="R26c875b4db5a47e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="Rd6378cf653b84ed8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实验登记" sheetId="2" r:id="R262bfb0067f74339"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="Ra651f1c1d478496f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -693,7 +693,7 @@
         <x:v>总实验数</x:v>
       </x:c>
       <x:c r="B4" s="15" t="n">
-        <x:v>17</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -701,7 +701,7 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="B5" s="15" t="n">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -709,7 +709,7 @@
         <x:v>计划中</x:v>
       </x:c>
       <x:c r="B6" s="15" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -717,7 +717,7 @@
         <x:v>等待结论</x:v>
       </x:c>
       <x:c r="B7" s="15" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -725,7 +725,7 @@
         <x:v>最新登记日期</x:v>
       </x:c>
       <x:c r="B8" s="18" t="n">
-        <x:v>46265.11111111111</x:v>
+        <x:v>46265.16001157407</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -733,7 +733,7 @@
         <x:v>登记来源</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>configs/experiments/*.yaml + outputs/&lt;实验ID&gt;/runs/*（E0014–E0017 已登记）</x:v>
+        <x:v>configs/experiments/*.yaml + outputs/&lt;实验ID&gt;/runs/*（E0014–E0018 已登记）</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26" customHeight="1">
@@ -3513,17 +3513,161 @@
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="F21" s="53"/>
-      <x:c r="AO21" s="55"/>
-      <x:c r="AP21" s="55"/>
-      <x:c r="AQ21" s="55"/>
-      <x:c r="AR21" s="55"/>
-      <x:c r="AS21" s="55"/>
-      <x:c r="AT21" s="55"/>
-      <x:c r="AU21" s="55"/>
-      <x:c r="AV21" s="55"/>
-      <x:c r="AW21" s="55"/>
-      <x:c r="AX21" s="55"/>
+      <x:c r="A21" t="str">
+        <x:v>E0018</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>gcn_gru_dynamic_only_mse_w1_control_v1</x:v>
+      </x:c>
+      <x:c r="C21" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>sequence</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>AWAITING_CONCLUSION</x:v>
+      </x:c>
+      <x:c r="F21" s="53" t="n">
+        <x:v>46265.148877314816</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>E0012</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>在E0012无边重建的动态压力测试中，将差分与全程方差损失从3:3同步缩放为1:1，整体损失尺度是否会改变dFC动态塌缩与验证表现</x:v>
+      </x:c>
+      <x:c r="I21" t="str">
+        <x:v>若E0018与E0012的动态诊断接近，则3:3与1:1的整体缩放不改变核心结论，后续可固定总尺度而只调两项损失比例；若明显不同，则总体梯度尺度是重要优化因素。</x:v>
+      </x:c>
+      <x:c r="J21" t="str">
+        <x:v>保持E0012的无边重建、GCN+GRU、冻结decoder和50 epoch设置，仅将MSE损失由3·L_diff + 3·L_var改为1·L_diff + 1·L_var</x:v>
+      </x:c>
+      <x:c r="K21" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="L21" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M21" t="str">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N21" t="str">
+        <x:v>gru</x:v>
+      </x:c>
+      <x:c r="O21" t="str">
+        <x:v>hcp_gcn</x:v>
+      </x:c>
+      <x:c r="P21" t="str">
+        <x:v>e0003_reconstruction_decoder</x:v>
+      </x:c>
+      <x:c r="Q21" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R21" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="S21" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T21" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="U21" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="V21" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W21" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="X21" s="49" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y21" t="str">
+        <x:v>mse</x:v>
+      </x:c>
+      <x:c r="Z21" t="str">
+        <x:v>mse：L = 1·L_diff + 1·L_var</x:v>
+      </x:c>
+      <x:c r="AA21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AB21" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AC21"/>
+      <x:c r="AD21" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="AE21"/>
+      <x:c r="AF21"/>
+      <x:c r="AG21"/>
+      <x:c r="AH21"/>
+      <x:c r="AI21" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="AJ21" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AK21" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="AL21" t="n">
+        <x:v>0.0003</x:v>
+      </x:c>
+      <x:c r="AM21" t="n">
+        <x:v>0.0001</x:v>
+      </x:c>
+      <x:c r="AN21" t="str">
+        <x:v>objective_loss</x:v>
+      </x:c>
+      <x:c r="AO21" s="55" t="n">
+        <x:v>0.012745602975917768</x:v>
+      </x:c>
+      <x:c r="AP21" s="55" t="str">
+        <x:v>E0018-s42-20260831T033422Z-9e36157</x:v>
+      </x:c>
+      <x:c r="AQ21" s="55" t="str">
+        <x:v>COMPLETED</x:v>
+      </x:c>
+      <x:c r="AR21" s="55" t="n">
+        <x:v>2.458643065223211</x:v>
+      </x:c>
+      <x:c r="AS21" s="55" t="n">
+        <x:v>0.470785759106467</x:v>
+      </x:c>
+      <x:c r="AT21" s="55" t="n">
+        <x:v>-0.006210885091432034</x:v>
+      </x:c>
+      <x:c r="AU21" s="55" t="n">
+        <x:v>0.009545637465589032</x:v>
+      </x:c>
+      <x:c r="AV21" s="55" t="n">
+        <x:v>0.043030444202543816</x:v>
+      </x:c>
+      <x:c r="AW21" s="55" t="n">
+        <x:v>0.08815911086865619</x:v>
+      </x:c>
+      <x:c r="AX21" s="55" t="n">
+        <x:v>0.5578604483906227</x:v>
+      </x:c>
+      <x:c r="AY21" t="str">
+        <x:v>训练、验证与动态审计已完成：non-overlap temporal std ratio=1.016，difference std ratio=0.088，difference temporal Pearson=-0.0002。</x:v>
+      </x:c>
+      <x:c r="AZ21" t="str">
+        <x:v>与E0012比较共同缩放3:3→1:1对动态诊断的影响；不得比较objective_loss绝对值。</x:v>
+      </x:c>
+      <x:c r="BA21" t="str">
+        <x:v>configs/experiments/E0018_gcn_gru_dynamic_only_mse_w1_control_v1.yaml</x:v>
+      </x:c>
+      <x:c r="BB21" t="str">
+        <x:v>e1a24d8a0d35ccf30d4b49ba9b0fa21fa82a8efcd8e7d81b4dc49635a8f0596c</x:v>
+      </x:c>
+      <x:c r="BC21" t="str">
+        <x:v>固定完成50个epoch且不查看测试集；与E0012在验证集比较temporal_std_ratio、difference_std_ratio、difference_temporal_pearson、dynamic_amplitude_mae、difference_mse、MSE、long_residual_pearson和FCD。不得以objective_loss绝对值比较，因为该值会随共同缩放的损失系数改变。</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="F22" s="53"/>
@@ -5870,7 +6014,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R973a768845d14348"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7bfa88502564e49"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
artifacts: publish E0019-E0021 loss ratio sweep
</commit_message>
<xml_diff>
--- a/outputs/experiment_registry_excel_20260828/HCP_dFC_实验登记册.xlsx
+++ b/outputs/experiment_registry_excel_20260828/HCP_dFC_实验登记册.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="Rd6378cf653b84ed8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实验登记" sheetId="2" r:id="R262bfb0067f74339"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="Ra651f1c1d478496f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="1" r:id="R676ba090426d4f28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="实验登记" sheetId="2" r:id="R72a185048e064346"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" r:id="R1adcd38ffb93496c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -693,7 +693,7 @@
         <x:v>总实验数</x:v>
       </x:c>
       <x:c r="B4" s="15" t="n">
-        <x:v>18</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -701,7 +701,7 @@
         <x:v>已完成</x:v>
       </x:c>
       <x:c r="B5" s="15" t="n">
-        <x:v>15</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -717,7 +717,7 @@
         <x:v>等待结论</x:v>
       </x:c>
       <x:c r="B7" s="15" t="n">
-        <x:v>16</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -725,7 +725,7 @@
         <x:v>最新登记日期</x:v>
       </x:c>
       <x:c r="B8" s="18" t="n">
-        <x:v>46265.16001157407</x:v>
+        <x:v>46265.316157407404</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -733,7 +733,7 @@
         <x:v>登记来源</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>configs/experiments/*.yaml + outputs/&lt;实验ID&gt;/runs/*（E0014–E0018 已登记）</x:v>
+        <x:v>configs/experiments/*.yaml + outputs/&lt;实验ID&gt;/runs/*（E0014–E0021 已登记）</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="26" customHeight="1">
@@ -3670,43 +3670,475 @@
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="F22" s="53"/>
-      <x:c r="AO22" s="55"/>
-      <x:c r="AP22" s="55"/>
-      <x:c r="AQ22" s="55"/>
-      <x:c r="AR22" s="55"/>
-      <x:c r="AS22" s="55"/>
-      <x:c r="AT22" s="55"/>
-      <x:c r="AU22" s="55"/>
-      <x:c r="AV22" s="55"/>
-      <x:c r="AW22" s="55"/>
-      <x:c r="AX22" s="55"/>
+      <x:c r="A22" t="str">
+        <x:v>E0019</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>gcn_gru_dynamic_only_mse_diff_bias_v1</x:v>
+      </x:c>
+      <x:c r="C22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>sequence</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>AWAITING_CONCLUSION</x:v>
+      </x:c>
+      <x:c r="F22" s="53" t="n">
+        <x:v>46265.27394675926</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>E0018</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>在E0018的1:1动态损失基准上，提高差分项相对权重是否能优先恢复dFC变化方向与时间细节</x:v>
+      </x:c>
+      <x:c r="I22" t="str">
+        <x:v>差分项偏重可能改善逐窗变化方向，但由于方差约束减弱，动态幅值和低频功率仍可能不足</x:v>
+      </x:c>
+      <x:c r="J22" t="str">
+        <x:v>保持E0018总动态损失权重为2，仅将权重改为1.5·L_diff + 0.5·L_var</x:v>
+      </x:c>
+      <x:c r="K22" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="L22" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M22" t="str">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N22" t="str">
+        <x:v>gru</x:v>
+      </x:c>
+      <x:c r="O22" t="str">
+        <x:v>hcp_gcn</x:v>
+      </x:c>
+      <x:c r="P22" t="str">
+        <x:v>e0003_reconstruction_decoder</x:v>
+      </x:c>
+      <x:c r="Q22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R22" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="S22" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T22" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="U22" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="V22" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W22" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="X22" s="49" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y22" t="str">
+        <x:v>mse</x:v>
+      </x:c>
+      <x:c r="Z22" t="str">
+        <x:v>mse：L = 1.5·L_diff + 0.5·L_var</x:v>
+      </x:c>
+      <x:c r="AA22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AB22" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="AC22"/>
+      <x:c r="AD22" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="AE22"/>
+      <x:c r="AF22"/>
+      <x:c r="AG22"/>
+      <x:c r="AH22"/>
+      <x:c r="AI22" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="AJ22" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AK22" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="AL22" t="n">
+        <x:v>0.0003</x:v>
+      </x:c>
+      <x:c r="AM22" t="n">
+        <x:v>0.0001</x:v>
+      </x:c>
+      <x:c r="AN22" t="str">
+        <x:v>objective_loss</x:v>
+      </x:c>
+      <x:c r="AO22" s="55" t="n">
+        <x:v>0.01589634575987164</x:v>
+      </x:c>
+      <x:c r="AP22" s="55" t="str">
+        <x:v>E0019-s42-20260831T063429Z-3693165</x:v>
+      </x:c>
+      <x:c r="AQ22" s="55" t="str">
+        <x:v>COMPLETED</x:v>
+      </x:c>
+      <x:c r="AR22" s="55" t="n">
+        <x:v>2.516108270687393</x:v>
+      </x:c>
+      <x:c r="AS22" s="55" t="n">
+        <x:v>0.47846571572973756</x:v>
+      </x:c>
+      <x:c r="AT22" s="55" t="n">
+        <x:v>-0.00823612254749559</x:v>
+      </x:c>
+      <x:c r="AU22" s="55" t="n">
+        <x:v>0.009512066027691847</x:v>
+      </x:c>
+      <x:c r="AV22" s="55" t="n">
+        <x:v>0.04307422466293166</x:v>
+      </x:c>
+      <x:c r="AW22" s="55" t="n">
+        <x:v>0.09024763475113277</x:v>
+      </x:c>
+      <x:c r="AX22" s="55" t="n">
+        <x:v>0.5117017148604875</x:v>
+      </x:c>
+      <x:c r="AY22" t="str">
+        <x:v>验证MSE=2.5161，动态幅值MAE=0.0902；non-overlap temporal std ratio=0.974，difference std ratio=0.065，difference temporal Pearson=-0.0010，FCD=0.5117。与E0018比较待统一判定。</x:v>
+      </x:c>
+      <x:c r="AZ22" t="str">
+        <x:v>与E0018比较动态指标；若变化方向/细节不改善，不保留差分偏重。</x:v>
+      </x:c>
+      <x:c r="BA22" t="str">
+        <x:v>configs/experiments/E0019_gcn_gru_dynamic_only_mse_diff_bias_v1.yaml</x:v>
+      </x:c>
+      <x:c r="BB22" t="str">
+        <x:v>9c3e4d40bd365a10a7159b30052cc5d65eb6ecaec6a05766ad2e61478f4141c7</x:v>
+      </x:c>
+      <x:c r="BC22" t="str">
+        <x:v>固定完成50个epoch且不查看测试集；与E0018比较non-overlap动态幅值、差分标准差比、差分时间相关、频段功率、MSE、长程残差相关和FCD。不得仅按objective_loss绝对值比较。</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="F23" s="53"/>
-      <x:c r="AO23" s="55"/>
-      <x:c r="AP23" s="55"/>
-      <x:c r="AQ23" s="55"/>
-      <x:c r="AR23" s="55"/>
-      <x:c r="AS23" s="55"/>
-      <x:c r="AT23" s="55"/>
-      <x:c r="AU23" s="55"/>
-      <x:c r="AV23" s="55"/>
-      <x:c r="AW23" s="55"/>
-      <x:c r="AX23" s="55"/>
+      <x:c r="A23" t="str">
+        <x:v>E0020</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>gcn_gru_dynamic_only_mse_balanced_v1</x:v>
+      </x:c>
+      <x:c r="C23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>sequence</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>AWAITING_CONCLUSION</x:v>
+      </x:c>
+      <x:c r="F23" s="53" t="n">
+        <x:v>46265.289502314816</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>E0018</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>在E0018的1:1动态损失基准上，提高方差项相对权重并平衡两项实际贡献，能否改善dFC动态幅值</x:v>
+      </x:c>
+      <x:c r="I23" t="str">
+        <x:v>由于E0018中原始差分损失约为方差损失的3倍，0.5:1.5的权重可使两项实际优化贡献接近，从而改善动态幅值而不显著损失时间细节</x:v>
+      </x:c>
+      <x:c r="J23" t="str">
+        <x:v>保持E0018总动态损失权重为2，将权重改为0.5·L_diff + 1.5·L_var，使两项原始数值贡献近似平衡</x:v>
+      </x:c>
+      <x:c r="K23" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="L23" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M23" t="str">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N23" t="str">
+        <x:v>gru</x:v>
+      </x:c>
+      <x:c r="O23" t="str">
+        <x:v>hcp_gcn</x:v>
+      </x:c>
+      <x:c r="P23" t="str">
+        <x:v>e0003_reconstruction_decoder</x:v>
+      </x:c>
+      <x:c r="Q23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R23" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="S23" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T23" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="U23" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="V23" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W23" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="X23" s="49" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y23" t="str">
+        <x:v>mse</x:v>
+      </x:c>
+      <x:c r="Z23" t="str">
+        <x:v>mse：L = 0.5·L_diff + 1.5·L_var</x:v>
+      </x:c>
+      <x:c r="AA23" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AB23" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
+      <x:c r="AC23"/>
+      <x:c r="AD23" t="n">
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="AE23"/>
+      <x:c r="AF23"/>
+      <x:c r="AG23"/>
+      <x:c r="AH23"/>
+      <x:c r="AI23" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="AJ23" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AK23" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="AL23" t="n">
+        <x:v>0.0003</x:v>
+      </x:c>
+      <x:c r="AM23" t="n">
+        <x:v>0.0001</x:v>
+      </x:c>
+      <x:c r="AN23" t="str">
+        <x:v>objective_loss</x:v>
+      </x:c>
+      <x:c r="AO23" s="55" t="n">
+        <x:v>0.009469563966687721</x:v>
+      </x:c>
+      <x:c r="AP23" s="55" t="str">
+        <x:v>E0020-s42-20260831T065652Z-3693165</x:v>
+      </x:c>
+      <x:c r="AQ23" s="55" t="str">
+        <x:v>COMPLETED</x:v>
+      </x:c>
+      <x:c r="AR23" s="55" t="n">
+        <x:v>2.147602123550222</x:v>
+      </x:c>
+      <x:c r="AS23" s="55" t="n">
+        <x:v>0.4156641788497756</x:v>
+      </x:c>
+      <x:c r="AT23" s="55" t="n">
+        <x:v>-0.007462341473968346</x:v>
+      </x:c>
+      <x:c r="AU23" s="55" t="n">
+        <x:v>0.009577228292775682</x:v>
+      </x:c>
+      <x:c r="AV23" s="55" t="n">
+        <x:v>0.042273088853476165</x:v>
+      </x:c>
+      <x:c r="AW23" s="55" t="n">
+        <x:v>0.08688467698572558</x:v>
+      </x:c>
+      <x:c r="AX23" s="55" t="n">
+        <x:v>0.37962556973429795</x:v>
+      </x:c>
+      <x:c r="AY23" t="str">
+        <x:v>验证MSE=2.1476，动态幅值MAE=0.0869；non-overlap temporal std ratio=0.795，difference std ratio=0.071，difference temporal Pearson=0.0019，FCD=0.3796。与E0018比较待统一判定。</x:v>
+      </x:c>
+      <x:c r="AZ23" t="str">
+        <x:v>与E0018比较；若幅值改善但时间方差仍&lt;1，继续做比值细扫或引入直接幅值约束。</x:v>
+      </x:c>
+      <x:c r="BA23" t="str">
+        <x:v>configs/experiments/E0020_gcn_gru_dynamic_only_mse_balanced_v1.yaml</x:v>
+      </x:c>
+      <x:c r="BB23" t="str">
+        <x:v>8e6d26643a6e96bfdfbf67a2b8229da125f19ab6457b5c28a34c3ad22279ff63</x:v>
+      </x:c>
+      <x:c r="BC23" t="str">
+        <x:v>固定完成50个epoch且不查看测试集；与E0018比较non-overlap动态幅值、差分标准差比、差分时间相关、频段功率、MSE、长程残差相关和FCD。不得仅按objective_loss绝对值比较。</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="F24" s="53"/>
-      <x:c r="AO24" s="55"/>
-      <x:c r="AP24" s="55"/>
-      <x:c r="AQ24" s="55"/>
-      <x:c r="AR24" s="55"/>
-      <x:c r="AS24" s="55"/>
-      <x:c r="AT24" s="55"/>
-      <x:c r="AU24" s="55"/>
-      <x:c r="AV24" s="55"/>
-      <x:c r="AW24" s="55"/>
-      <x:c r="AX24" s="55"/>
+      <x:c r="A24" t="str">
+        <x:v>E0021</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>gcn_gru_dynamic_only_mse_variance_bias_v1</x:v>
+      </x:c>
+      <x:c r="C24" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>sequence</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>AWAITING_CONCLUSION</x:v>
+      </x:c>
+      <x:c r="F24" s="53" t="n">
+        <x:v>46265.30533564815</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>E0018</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>在E0018的1:1动态损失基准上，明显提高方差项相对权重能否进一步解除dFC动态幅值塌缩</x:v>
+      </x:c>
+      <x:c r="I24" t="str">
+        <x:v>方差项偏重可能进一步拉高总体动态幅值，但若缺少足够的差分约束，时间顺序、变化方向和细节重建可能恶化</x:v>
+      </x:c>
+      <x:c r="J24" t="str">
+        <x:v>保持E0018总动态损失权重为2，仅将权重改为0.2·L_diff + 1.8·L_var</x:v>
+      </x:c>
+      <x:c r="K24" t="n">
+        <x:v>83</x:v>
+      </x:c>
+      <x:c r="L24" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="M24" t="str">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="N24" t="str">
+        <x:v>gru</x:v>
+      </x:c>
+      <x:c r="O24" t="str">
+        <x:v>hcp_gcn</x:v>
+      </x:c>
+      <x:c r="P24" t="str">
+        <x:v>e0003_reconstruction_decoder</x:v>
+      </x:c>
+      <x:c r="Q24" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R24" t="str">
+        <x:v>none</x:v>
+      </x:c>
+      <x:c r="S24" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="T24" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="U24" t="n">
+        <x:v>256</x:v>
+      </x:c>
+      <x:c r="V24" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="W24" t="n">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="X24" s="49" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y24" t="str">
+        <x:v>mse</x:v>
+      </x:c>
+      <x:c r="Z24" t="str">
+        <x:v>mse：L = 0.2·L_diff + 1.8·L_var</x:v>
+      </x:c>
+      <x:c r="AA24" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AB24" t="n">
+        <x:v>0.2</x:v>
+      </x:c>
+      <x:c r="AC24"/>
+      <x:c r="AD24" t="n">
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="AE24"/>
+      <x:c r="AF24"/>
+      <x:c r="AG24"/>
+      <x:c r="AH24"/>
+      <x:c r="AI24" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="AJ24" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="AK24" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="AL24" t="n">
+        <x:v>0.0003</x:v>
+      </x:c>
+      <x:c r="AM24" t="n">
+        <x:v>0.0001</x:v>
+      </x:c>
+      <x:c r="AN24" t="str">
+        <x:v>objective_loss</x:v>
+      </x:c>
+      <x:c r="AO24" s="55" t="n">
+        <x:v>0.007519746694383742</x:v>
+      </x:c>
+      <x:c r="AP24" s="55" t="str">
+        <x:v>E0021-s42-20260831T071941Z-3693165</x:v>
+      </x:c>
+      <x:c r="AQ24" s="55" t="str">
+        <x:v>COMPLETED</x:v>
+      </x:c>
+      <x:c r="AR24" s="55" t="n">
+        <x:v>2.27552496783341</x:v>
+      </x:c>
+      <x:c r="AS24" s="55" t="n">
+        <x:v>0.3827253485782237</x:v>
+      </x:c>
+      <x:c r="AT24" s="55" t="n">
+        <x:v>-0.005729638500016807</x:v>
+      </x:c>
+      <x:c r="AU24" s="55" t="n">
+        <x:v>0.009907352667349049</x:v>
+      </x:c>
+      <x:c r="AV24" s="55" t="n">
+        <x:v>0.042021168148310126</x:v>
+      </x:c>
+      <x:c r="AW24" s="55" t="n">
+        <x:v>0.07688354205670236</x:v>
+      </x:c>
+      <x:c r="AX24" s="55" t="n">
+        <x:v>0.32112975833536705</x:v>
+      </x:c>
+      <x:c r="AY24" t="str">
+        <x:v>验证MSE=2.2755，动态幅值MAE=0.0769；non-overlap temporal std ratio=0.503，difference std ratio=0.071，difference temporal Pearson=0.0001，FCD=0.3211。与E0018比较待统一判定。</x:v>
+      </x:c>
+      <x:c r="AZ24" t="str">
+        <x:v>与E0018比较；重点核查幅值、FCD和中低频功率，必要时回到1:1做更细网格。</x:v>
+      </x:c>
+      <x:c r="BA24" t="str">
+        <x:v>configs/experiments/E0021_gcn_gru_dynamic_only_mse_variance_bias_v1.yaml</x:v>
+      </x:c>
+      <x:c r="BB24" t="str">
+        <x:v>947fc020ededcfe2265e12295b21702709bc591a97f57c63e6372a3b7b2b3282</x:v>
+      </x:c>
+      <x:c r="BC24" t="str">
+        <x:v>固定完成50个epoch且不查看测试集；与E0018比较non-overlap动态幅值、差分标准差比、差分时间相关、频段功率、MSE、长程残差相关和FCD。不得仅按objective_loss绝对值比较。</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="F25" s="53"/>
@@ -6014,7 +6446,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7bfa88502564e49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6562db9b39844e29"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>